<commit_message>
addressing issue: golden port will not be override
</commit_message>
<xml_diff>
--- a/Testkit_Q1_PRN222/Q11/Environment.xlsx
+++ b/Testkit_Q1_PRN222/Q11/Environment.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\1\Downloads\QuestionQ1_FA25\Testkit_Q1_PRN222\Q11\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\School\NET\auto-grading\Testkit_Q1_PRN222\Q11\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C881A042-9EFF-440D-84BF-E543FDDC18AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD47EE05-BA0F-42C7-A6F9-91A518B793BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -232,7 +232,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -244,7 +244,7 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -264,7 +264,7 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
-      <name val="Aptos Narrow"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -881,13 +881,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B25"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.09765625" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.77734375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="42.88671875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="10.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="9.109375" style="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.109375" style="1"/>
+    <col min="1" max="1" width="30.796875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="42.8984375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="10.69921875" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="9.09765625" style="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.09765625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -935,7 +935,7 @@
         <v>9</v>
       </c>
       <c r="B6" s="19">
-        <v>4000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -943,7 +943,7 @@
         <v>10</v>
       </c>
       <c r="B7" s="21">
-        <v>4000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -1018,7 +1018,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="18" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
         <v>25</v>
       </c>
@@ -1089,14 +1089,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89A83C95-3B80-4231-A2A3-554283AC2A02}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.6640625" style="6" customWidth="1"/>
-    <col min="2" max="2" width="37.21875" style="7" customWidth="1"/>
+    <col min="1" max="1" width="21.69921875" style="6" customWidth="1"/>
+    <col min="2" max="2" width="37.19921875" style="7" customWidth="1"/>
     <col min="3" max="3" width="66" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>35</v>
       </c>
@@ -1107,7 +1107,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="27" t="s">
         <v>38</v>
       </c>
@@ -1118,7 +1118,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="27"/>
       <c r="B3" s="3" t="s">
         <v>41</v>
@@ -1127,7 +1127,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="27"/>
       <c r="B4" s="3" t="s">
         <v>43</v>
@@ -1136,7 +1136,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="27"/>
       <c r="B5" s="3" t="s">
         <v>45</v>
@@ -1145,7 +1145,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="27"/>
       <c r="B6" s="3" t="s">
         <v>47</v>
@@ -1154,7 +1154,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="28" t="s">
         <v>49</v>
       </c>
@@ -1165,28 +1165,28 @@
         <v>51</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="27"/>
       <c r="B8" s="3" t="s">
         <v>52</v>
       </c>
       <c r="C8" s="3"/>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="27"/>
       <c r="B9" s="3" t="s">
         <v>53</v>
       </c>
       <c r="C9" s="3"/>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="27"/>
       <c r="B10" s="3" t="s">
         <v>54</v>
       </c>
       <c r="C10" s="3"/>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="29"/>
       <c r="B11" s="4" t="s">
         <v>55</v>
@@ -1205,12 +1205,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66E063F4-52D0-4D9A-9D12-41E03025E950}">
   <dimension ref="A1:B23"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.8984375" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7" style="22" customWidth="1"/>
-    <col min="2" max="2" width="27.21875" style="22" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.88671875" style="22" customWidth="1"/>
-    <col min="4" max="16384" width="8.88671875" style="22"/>
+    <col min="2" max="2" width="27.19921875" style="22" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.8984375" style="22" customWidth="1"/>
+    <col min="4" max="16384" width="8.8984375" style="22"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -1247,12 +1247,12 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B6" s="22">
-        <v>4000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B7" s="22">
-        <v>4000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>